<commit_message>
chore: update binary files and remove obsolete Excel document
</commit_message>
<xml_diff>
--- a/All_Prices.xlsx
+++ b/All_Prices.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yadmitrieva/EPL Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C542C88D-1C2F-A04C-AF53-A14854371457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D11D6E-D733-2144-963D-9AC5BE303601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="820" windowWidth="30240" windowHeight="17440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="30240" windowHeight="17440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Admin" sheetId="5" r:id="rId1"/>
@@ -839,125 +839,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yy"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="1"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1408,6 +1289,125 @@
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy;@"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yy"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="1"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1422,27 +1422,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0F118954-90FD-1D49-8627-2A87DB299C4D}" name="T_PriceListsDatabase" displayName="T_PriceListsDatabase" ref="A1:P99" totalsRowShown="0" headerRowDxfId="25">
-  <autoFilter ref="A1:P99" xr:uid="{0F118954-90FD-1D49-8627-2A87DB299C4D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0F118954-90FD-1D49-8627-2A87DB299C4D}" name="T_PriceListsDatabase" displayName="T_PriceListsDatabase" ref="A1:P99" totalsRowShown="0" headerRowDxfId="33">
+  <autoFilter ref="A1:P99" xr:uid="{0F118954-90FD-1D49-8627-2A87DB299C4D}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="V1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{37D2F902-ABD9-4643-A4D7-B5B95F8EB3DD}" name="SAP Plant"/>
-    <tableColumn id="2" xr3:uid="{5B3FAA56-8691-6B45-BE88-1FAD6CD79814}" name="Customer ref. SAP" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{371D5FE5-8C9A-EC43-BDB3-7F3A516D0026}" name="Effective" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{C5A79962-6221-1549-BAB4-FC8C5A183437}" name="Mailing date" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{CD814802-AC17-394B-824B-A91512F11E29}" name="Customer Short Name" dataDxfId="21">
+    <tableColumn id="2" xr3:uid="{5B3FAA56-8691-6B45-BE88-1FAD6CD79814}" name="Customer ref. SAP" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{371D5FE5-8C9A-EC43-BDB3-7F3A516D0026}" name="Effective" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{C5A79962-6221-1549-BAB4-FC8C5A183437}" name="Mailing date" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{CD814802-AC17-394B-824B-A91512F11E29}" name="Customer Short Name" dataDxfId="29">
       <calculatedColumnFormula>_xlfn.XLOOKUP('Prices Database'!B2,'Customers Masterdata'!F:F,'Customers Masterdata'!G:G)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{35843D4F-3CF9-5A45-94C4-C2D637FC48E1}" name="Price List Version" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{D909CC7A-A93A-144B-A2AE-682919516B1F}" name="Comments about Changes" dataDxfId="19"/>
-    <tableColumn id="15" xr3:uid="{803EFC74-00E4-464C-91D8-8542A8D43EC2}" name="Price Type (Discount, Net Price)" dataDxfId="18"/>
-    <tableColumn id="16" xr3:uid="{073928F4-7D0B-BB49-AEE6-06E3D09F786E}" name="If Type Discount - Discount %" dataDxfId="17"/>
-    <tableColumn id="8" xr3:uid="{19E42D72-2648-484B-8CF2-B93EA577FF36}" name="Price List ID" dataDxfId="16">
+    <tableColumn id="6" xr3:uid="{35843D4F-3CF9-5A45-94C4-C2D637FC48E1}" name="Price List Version" dataDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{D909CC7A-A93A-144B-A2AE-682919516B1F}" name="Comments about Changes" dataDxfId="27"/>
+    <tableColumn id="15" xr3:uid="{803EFC74-00E4-464C-91D8-8542A8D43EC2}" name="Price Type (Discount, Net Price)" dataDxfId="26"/>
+    <tableColumn id="16" xr3:uid="{073928F4-7D0B-BB49-AEE6-06E3D09F786E}" name="If Type Discount - Discount %" dataDxfId="25"/>
+    <tableColumn id="8" xr3:uid="{19E42D72-2648-484B-8CF2-B93EA577FF36}" name="Price List ID" dataDxfId="24">
       <calculatedColumnFormula>B2&amp;C2&amp;D2&amp;F2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="9" xr3:uid="{4FB4E62E-D1DE-7744-BE1C-C17981BFA9AE}" name="Product type"/>
-    <tableColumn id="10" xr3:uid="{3CA5389E-BE54-514B-BBCB-ECBF466B186F}" name="RIP code" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{3CA5389E-BE54-514B-BBCB-ECBF466B186F}" name="RIP code" dataDxfId="23"/>
     <tableColumn id="11" xr3:uid="{C0411C6D-51D5-4A4F-8872-BC47F7B10E29}" name="Product"/>
-    <tableColumn id="12" xr3:uid="{96C25DB5-B98C-FA40-B263-F9612D0DADE1}" name="Net price_x000a_(Currency / Unit)" dataDxfId="14"/>
+    <tableColumn id="12" xr3:uid="{96C25DB5-B98C-FA40-B263-F9612D0DADE1}" name="Net price_x000a_(Currency / Unit)" dataDxfId="22"/>
     <tableColumn id="13" xr3:uid="{FE678BD4-6DEE-7B47-B7BA-64578B01D1A7}" name="Currency"/>
     <tableColumn id="14" xr3:uid="{18D3A197-DB24-144D-940B-A2D922C84EEA}" name="Unit"/>
   </tableColumns>
@@ -1457,7 +1463,7 @@
     <tableColumn id="1" xr3:uid="{C394DC01-2FA5-F249-8E27-593C8E0CC130}" name="Packagin Version"/>
     <tableColumn id="2" xr3:uid="{235AF419-5F84-8F45-8F40-4227D19A3017}" name="Product Type"/>
     <tableColumn id="4" xr3:uid="{2492B6A6-ECAD-B944-9286-1D10F97121C1}" name="Packaging Name"/>
-    <tableColumn id="5" xr3:uid="{15301E65-3DD2-6D42-98FE-D9684530DE40}" name="Price" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{15301E65-3DD2-6D42-98FE-D9684530DE40}" name="Price" dataDxfId="21"/>
     <tableColumn id="6" xr3:uid="{38E11289-FFED-F242-8D66-3814249EB7CB}" name="Currency"/>
     <tableColumn id="7" xr3:uid="{B03AE9A3-266E-E84E-A2EF-1EC53CADA514}" name="Unit"/>
   </tableColumns>
@@ -1472,7 +1478,7 @@
     <tableColumn id="1" xr3:uid="{548B632C-CB06-6149-BFED-10326A4592F6}" name="Packagin Version"/>
     <tableColumn id="2" xr3:uid="{E7552D57-4470-7049-901C-65B811D82275}" name="Product Type"/>
     <tableColumn id="3" xr3:uid="{EC1D7A85-3113-0345-A020-6F4A505D0616}" name="Packaging Name"/>
-    <tableColumn id="4" xr3:uid="{5EFFAEFC-4F74-0446-844E-7CED7F985D3B}" name="Price" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{5EFFAEFC-4F74-0446-844E-7CED7F985D3B}" name="Price" dataDxfId="20"/>
     <tableColumn id="5" xr3:uid="{A14B6A73-05FD-684E-B7F2-CB1A0E156CAF}" name="Currency"/>
     <tableColumn id="6" xr3:uid="{5E311707-2C84-4840-9044-C36D000DAEC6}" name="Unit"/>
   </tableColumns>
@@ -1481,7 +1487,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{018A20AE-9210-2043-B769-6227B8627523}" name="T_CustomerMasterdata" displayName="T_CustomerMasterdata" ref="A1:T3" totalsRowShown="0" headerRowDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{018A20AE-9210-2043-B769-6227B8627523}" name="T_CustomerMasterdata" displayName="T_CustomerMasterdata" ref="A1:T3" totalsRowShown="0" headerRowDxfId="43">
   <autoFilter ref="A1:T3" xr:uid="{018A20AE-9210-2043-B769-6227B8627523}"/>
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{7EB59029-C014-3344-9B1E-D008A6B2DA3B}" name="Zone"/>
@@ -1489,22 +1495,22 @@
     <tableColumn id="3" xr3:uid="{A908BA89-C7CB-6B41-85D5-1C0DF4FB4D46}" name="Customer Type"/>
     <tableColumn id="4" xr3:uid="{B9BDA364-BF2D-F540-BCD6-07DD275210AC}" name="Comment on Business Model"/>
     <tableColumn id="5" xr3:uid="{B88C2814-DEC7-F84F-8661-43580C35894C}" name="Customer ref. type SAP"/>
-    <tableColumn id="6" xr3:uid="{2248B505-D962-1C43-B454-A4B8B178A3A3}" name="Customer ref. SAP" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{0D5F9FD0-FC01-4E48-A7BA-C4855FE9E8DF}" name="Customer Short Name" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{97C47538-7703-A249-BD86-0BB7284A02BA}" name="Customer Full Name" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{2248B505-D962-1C43-B454-A4B8B178A3A3}" name="Customer ref. SAP" dataDxfId="42"/>
+    <tableColumn id="7" xr3:uid="{0D5F9FD0-FC01-4E48-A7BA-C4855FE9E8DF}" name="Customer Short Name" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{97C47538-7703-A249-BD86-0BB7284A02BA}" name="Customer Full Name" dataDxfId="40"/>
     <tableColumn id="9" xr3:uid="{3584453D-FF07-2B42-9C37-5EEDB8A1F9D8}" name="Currency"/>
     <tableColumn id="10" xr3:uid="{2897689C-CFDA-FD43-93C5-8C5944728291}" name="Packagin Version"/>
-    <tableColumn id="11" xr3:uid="{D2EDF6D2-15D0-6747-AC2D-FEF45DEB9429}" name="Pice List Managed by" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{2220F48A-029C-2545-90A3-F30C56C520A6}" name="Customer SPOC" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{E58B7D03-8C98-B549-9F8C-13E8A39B9A7F}" name="Effective" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{61359FB1-0C15-9646-BC4E-8F4924D00884}" name="Mailing date" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{D2EDF6D2-15D0-6747-AC2D-FEF45DEB9429}" name="Pice List Managed by" dataDxfId="39"/>
+    <tableColumn id="12" xr3:uid="{2220F48A-029C-2545-90A3-F30C56C520A6}" name="Customer SPOC" dataDxfId="38"/>
+    <tableColumn id="13" xr3:uid="{E58B7D03-8C98-B549-9F8C-13E8A39B9A7F}" name="Effective" dataDxfId="37"/>
+    <tableColumn id="14" xr3:uid="{61359FB1-0C15-9646-BC4E-8F4924D00884}" name="Mailing date" dataDxfId="36"/>
     <tableColumn id="15" xr3:uid="{FAD338F2-73B5-D14D-A9DA-8A2B14C800D0}" name="Last Price List Version"/>
-    <tableColumn id="20" xr3:uid="{187403D4-6469-DC45-BA9B-16EA70F7835F}" name="Last Price List ID" dataDxfId="3">
+    <tableColumn id="20" xr3:uid="{187403D4-6469-DC45-BA9B-16EA70F7835F}" name="Last Price List ID" dataDxfId="35">
       <calculatedColumnFormula>T_CustomerMasterdata[[#This Row],[Customer ref. SAP]]&amp;T_CustomerMasterdata[[#This Row],[Effective]]&amp;T_CustomerMasterdata[[#This Row],[Mailing date]]&amp;T_CustomerMasterdata[[#This Row],[Last Price List Version]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{EC332BF1-4B64-5B43-BC9E-F79444DCF47A}" name="Mailing TO: Customer"/>
     <tableColumn id="17" xr3:uid="{9EBF1ECC-3E2A-3946-BB40-511666ABEA7E}" name="Internal COPY: SPOC + RZM + Other"/>
-    <tableColumn id="18" xr3:uid="{BA8B7E30-778E-CF43-8DDD-8E78FEC4DA23}" name="Internal COPY to: PBP (Costing manager)" dataDxfId="2" dataCellStyle="Hyperlink">
+    <tableColumn id="18" xr3:uid="{BA8B7E30-778E-CF43-8DDD-8E78FEC4DA23}" name="Internal COPY to: PBP (Costing manager)" dataDxfId="34" dataCellStyle="Hyperlink">
       <calculatedColumnFormula>V_Email_PBPCostingManager</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="19" xr3:uid="{4AC3D85B-5286-AD4D-A8BF-16A422922E85}" name="COPY to: PBP common mail box"/>
@@ -1514,30 +1520,30 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{08583D75-F5E0-9247-8420-043E947DF895}" name="Table_StandardEPL_USD" displayName="Table_StandardEPL_USD" ref="A1:F46" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42" tableBorderDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{08583D75-F5E0-9247-8420-043E947DF895}" name="Table_StandardEPL_USD" displayName="Table_StandardEPL_USD" ref="A1:F46" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18" tableBorderDxfId="17">
   <autoFilter ref="A1:F46" xr:uid="{08583D75-F5E0-9247-8420-043E947DF895}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{D5370C0F-EF1F-FE4E-823B-BC12FBF5E1D8}" name="Product type" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{AFD818D7-01BD-EA47-8510-CE3DB782DEF7}" name="RIP code" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{BA1D3757-D246-9A40-95A5-59035BC3596B}" name="Product" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{19A22FA5-1301-2048-A200-D2786122F32C}" name="Net price_x000a_(Currency / Unit)" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{3D9EC9B7-AFFB-064C-8969-D35D91D4911A}" name="Currency" dataDxfId="36"/>
-    <tableColumn id="6" xr3:uid="{132A2678-6F02-3B48-A3D3-9A7A1715C7E3}" name="Unit" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{D5370C0F-EF1F-FE4E-823B-BC12FBF5E1D8}" name="Product type" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{AFD818D7-01BD-EA47-8510-CE3DB782DEF7}" name="RIP code" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{BA1D3757-D246-9A40-95A5-59035BC3596B}" name="Product" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{19A22FA5-1301-2048-A200-D2786122F32C}" name="Net price_x000a_(Currency / Unit)" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{3D9EC9B7-AFFB-064C-8969-D35D91D4911A}" name="Currency" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{132A2678-6F02-3B48-A3D3-9A7A1715C7E3}" name="Unit" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C9FDDAA2-BE48-784E-9ADE-65BB176C5DFA}" name="Table_StandardEPL_EUR" displayName="Table_StandardEPL_EUR" ref="I1:N12" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33" tableBorderDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{C9FDDAA2-BE48-784E-9ADE-65BB176C5DFA}" name="Table_StandardEPL_EUR" displayName="Table_StandardEPL_EUR" ref="I1:N12" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="I1:N12" xr:uid="{C9FDDAA2-BE48-784E-9ADE-65BB176C5DFA}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{E5F45572-BC3D-E84C-819A-8A61994AFC61}" name="Product type" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{2464CE3D-2F29-3641-80B9-F388FE026E6C}" name="RIP code" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{B9359043-9086-8F4B-AED6-7C5C27FB0A7D}" name="Product" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{8658424D-4B49-EA49-82C4-7494A9E30DA0}" name="Net price_x000a_(Currency / Unit)" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{A439F0F3-48F3-5B4B-A620-C67704060E10}" name="Currency" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{7F65394B-ED7C-6148-B52C-C9B1DADA10E5}" name="Unit" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{E5F45572-BC3D-E84C-819A-8A61994AFC61}" name="Product type" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{2464CE3D-2F29-3641-80B9-F388FE026E6C}" name="RIP code" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{B9359043-9086-8F4B-AED6-7C5C27FB0A7D}" name="Product" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{8658424D-4B49-EA49-82C4-7494A9E30DA0}" name="Net price_x000a_(Currency / Unit)" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{A439F0F3-48F3-5B4B-A620-C67704060E10}" name="Currency" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{7F65394B-ED7C-6148-B52C-C9B1DADA10E5}" name="Unit" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3949,10 +3955,10 @@
         <v>58</v>
       </c>
       <c r="C43" s="19">
-        <v>45444</v>
+        <v>36527</v>
       </c>
       <c r="D43" s="19">
-        <v>45454</v>
+        <v>36526</v>
       </c>
       <c r="E43" s="5" t="str">
         <f>_xlfn.XLOOKUP('Prices Database'!B43,'Customers Masterdata'!F:F,'Customers Masterdata'!G:G)</f>
@@ -3972,7 +3978,7 @@
       </c>
       <c r="J43" s="5" t="str">
         <f t="shared" si="1"/>
-        <v>XXXXX14544445454V1</v>
+        <v>XXXXX13652736526V1</v>
       </c>
       <c r="K43" t="s">
         <v>14</v>
@@ -3993,7 +3999,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>165</v>
       </c>
@@ -4045,7 +4051,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>165</v>
       </c>
@@ -4097,7 +4103,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B46" s="3" t="s">
         <v>58</v>
       </c>
@@ -4146,7 +4152,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B47" s="3" t="s">
         <v>58</v>
       </c>
@@ -4195,7 +4201,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B48" s="3" t="s">
         <v>58</v>
       </c>
@@ -4244,7 +4250,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="49" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B49" s="3" t="s">
         <v>58</v>
       </c>
@@ -4293,7 +4299,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="50" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B50" s="3" t="s">
         <v>58</v>
       </c>
@@ -4342,7 +4348,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B51" s="3" t="s">
         <v>58</v>
       </c>
@@ -4391,7 +4397,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="52" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B52" s="3" t="s">
         <v>58</v>
       </c>
@@ -4440,7 +4446,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="53" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B53" s="3" t="s">
         <v>58</v>
       </c>
@@ -4489,7 +4495,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="54" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B54" s="3" t="s">
         <v>58</v>
       </c>
@@ -4538,7 +4544,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="55" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B55" s="3" t="s">
         <v>58</v>
       </c>
@@ -4587,7 +4593,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="56" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B56" s="3" t="s">
         <v>58</v>
       </c>
@@ -4636,7 +4642,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B57" s="3" t="s">
         <v>58</v>
       </c>
@@ -4685,7 +4691,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="58" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B58" s="3" t="s">
         <v>58</v>
       </c>
@@ -4734,7 +4740,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B59" s="3" t="s">
         <v>58</v>
       </c>
@@ -4783,7 +4789,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="60" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B60" s="3" t="s">
         <v>58</v>
       </c>
@@ -4832,7 +4838,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="61" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B61" s="3" t="s">
         <v>58</v>
       </c>
@@ -4881,7 +4887,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="62" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B62" s="3" t="s">
         <v>58</v>
       </c>
@@ -4930,7 +4936,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B63" s="3" t="s">
         <v>58</v>
       </c>
@@ -4979,7 +4985,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B64" s="3" t="s">
         <v>58</v>
       </c>
@@ -5028,7 +5034,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="65" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B65" s="3" t="s">
         <v>58</v>
       </c>
@@ -5077,7 +5083,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="66" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B66" s="3" t="s">
         <v>58</v>
       </c>
@@ -5126,7 +5132,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B67" s="3" t="s">
         <v>58</v>
       </c>
@@ -5175,7 +5181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="68" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B68" s="3" t="s">
         <v>58</v>
       </c>
@@ -5224,7 +5230,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="69" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B69" s="3" t="s">
         <v>58</v>
       </c>
@@ -5273,7 +5279,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="70" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B70" s="3" t="s">
         <v>58</v>
       </c>
@@ -5322,7 +5328,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B71" s="3" t="s">
         <v>58</v>
       </c>
@@ -5371,7 +5377,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="72" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B72" s="3" t="s">
         <v>58</v>
       </c>
@@ -5420,7 +5426,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="73" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B73" s="3" t="s">
         <v>58</v>
       </c>
@@ -5469,7 +5475,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="74" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B74" s="3" t="s">
         <v>58</v>
       </c>
@@ -5518,7 +5524,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B75" s="3" t="s">
         <v>58</v>
       </c>
@@ -5567,7 +5573,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="76" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B76" s="3" t="s">
         <v>58</v>
       </c>
@@ -5616,7 +5622,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B77" s="3" t="s">
         <v>58</v>
       </c>
@@ -5665,7 +5671,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="78" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B78" s="3" t="s">
         <v>58</v>
       </c>
@@ -5714,7 +5720,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="79" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B79" s="3" t="s">
         <v>58</v>
       </c>
@@ -5763,7 +5769,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="80" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B80" s="3" t="s">
         <v>58</v>
       </c>
@@ -5812,7 +5818,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B81" s="3" t="s">
         <v>58</v>
       </c>
@@ -5861,7 +5867,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B82" s="3" t="s">
         <v>58</v>
       </c>
@@ -5910,7 +5916,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B83" s="3" t="s">
         <v>58</v>
       </c>
@@ -5959,7 +5965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B84" s="3" t="s">
         <v>58</v>
       </c>
@@ -6008,7 +6014,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="85" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B85" s="3" t="s">
         <v>58</v>
       </c>
@@ -6057,7 +6063,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B86" s="3" t="s">
         <v>58</v>
       </c>
@@ -6106,7 +6112,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B87" s="3" t="s">
         <v>58</v>
       </c>
@@ -6155,7 +6161,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:16" hidden="1" x14ac:dyDescent="0.2">
       <c r="B88" s="3" t="s">
         <v>58</v>
       </c>
@@ -13437,12 +13443,36 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <DOC_TYPE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <REF_YEAR__x002f__ANNEE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">2023</REF_YEAR__x002f__ANNEE>
+    <PERIOD xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <DEPT_AUTOR xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <TARGET_AUDIENCE__x002f__DESTINATAIRE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <DOC_STATUS xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">Update Version/Version Actuelle</DOC_STATUS>
+    <Remark xmlns="7e83e573-fb93-452c-9f3b-7b87af48cc96" xsi:nil="true"/>
+    <DOC_LANGUAGE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">
+      <Value>French (France)</Value>
+    </DOC_LANGUAGE>
+    <MARKET__x002f__MARCHE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <TAG_2 xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <PRODUCT__x002f__RANGE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">
+      <Value>-</Value>
+    </PRODUCT__x002f__RANGE>
+    <IDENTIFICATION_REFERENCE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <DOMAIN xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <DOC_DESCRIPTION xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e83e573-fb93-452c-9f3b-7b87af48cc96">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+    <TAG_1 xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17130,42 +17160,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <DOC_TYPE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <REF_YEAR__x002f__ANNEE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">2023</REF_YEAR__x002f__ANNEE>
-    <PERIOD xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <DEPT_AUTOR xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <TARGET_AUDIENCE__x002f__DESTINATAIRE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <DOC_STATUS xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">Update Version/Version Actuelle</DOC_STATUS>
-    <Remark xmlns="7e83e573-fb93-452c-9f3b-7b87af48cc96" xsi:nil="true"/>
-    <DOC_LANGUAGE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">
-      <Value>French (France)</Value>
-    </DOC_LANGUAGE>
-    <MARKET__x002f__MARCHE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <TAG_2 xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <PRODUCT__x002f__RANGE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a">
-      <Value>-</Value>
-    </PRODUCT__x002f__RANGE>
-    <IDENTIFICATION_REFERENCE xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <DOMAIN xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <DOC_DESCRIPTION xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7e83e573-fb93-452c-9f3b-7b87af48cc96">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-    <TAG_1 xmlns="dc163805-5a8a-4bac-b0c0-60a9bfcd087a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08C24CE9-94B3-4210-8D15-1D41A580968E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F55DE33-C1A5-4F20-B814-5EC50C36FAFB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="dc163805-5a8a-4bac-b0c0-60a9bfcd087a"/>
+    <ds:schemaRef ds:uri="7e83e573-fb93-452c-9f3b-7b87af48cc96"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17190,12 +17199,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F55DE33-C1A5-4F20-B814-5EC50C36FAFB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08C24CE9-94B3-4210-8D15-1D41A580968E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="dc163805-5a8a-4bac-b0c0-60a9bfcd087a"/>
-    <ds:schemaRef ds:uri="7e83e573-fb93-452c-9f3b-7b87af48cc96"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>